<commit_message>
working decrement. adding ratio and tender logic
</commit_message>
<xml_diff>
--- a/Heuristic/data/real/Starting_point.xlsx
+++ b/Heuristic/data/real/Starting_point.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5e6b18ad1acc1266/Desktop/Vaccine_Tender/Heuristic/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5e6b18ad1acc1266/Desktop/Vaccine_Tender/Heuristic/data/real/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="94" documentId="13_ncr:1_{E4667220-B6D3-44CA-BB2C-7EE709A98D96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{86C9454B-4D20-4163-B5CD-9200BF1762CD}"/>
+  <xr:revisionPtr revIDLastSave="104" documentId="13_ncr:1_{E4667220-B6D3-44CA-BB2C-7EE709A98D96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7AAE704F-2B5C-4406-8534-45AFB0BB7DFF}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>

</xml_diff>

<commit_message>
updated starting inventory to match tenders; working tender code
</commit_message>
<xml_diff>
--- a/Heuristic/data/real/Starting_point.xlsx
+++ b/Heuristic/data/real/Starting_point.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5e6b18ad1acc1266/Desktop/Vaccine_Tender/Heuristic/data/real/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="104" documentId="13_ncr:1_{E4667220-B6D3-44CA-BB2C-7EE709A98D96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7AAE704F-2B5C-4406-8534-45AFB0BB7DFF}"/>
+  <xr:revisionPtr revIDLastSave="180" documentId="13_ncr:1_{E4667220-B6D3-44CA-BB2C-7EE709A98D96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BB51C906-A4DE-4E2A-A93D-9CAA728CF69A}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -186,12 +186,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="5">
+  <numFmts count="4">
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="0.00000E+00"/>
     <numFmt numFmtId="165" formatCode="0.000000E+00"/>
     <numFmt numFmtId="166" formatCode="0.000000"/>
-    <numFmt numFmtId="167" formatCode="0.000000%"/>
   </numFmts>
   <fonts count="6" x14ac:knownFonts="1">
     <font>
@@ -220,17 +219,17 @@
       <family val="3"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color rgb="FFCE9178"/>
-      <name val="Consolas"/>
-      <family val="3"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Consolas"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="2">
@@ -263,7 +262,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -276,19 +275,17 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -627,101 +624,101 @@
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="13" t="s">
+      <c r="A5" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="14">
-        <v>1</v>
-      </c>
-      <c r="C5" s="14">
+      <c r="B5" s="10">
+        <v>1</v>
+      </c>
+      <c r="C5" s="10">
         <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="13" t="s">
+      <c r="A6" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="14">
-        <v>1</v>
-      </c>
-      <c r="C6" s="14">
+      <c r="B6" s="10">
+        <v>1</v>
+      </c>
+      <c r="C6" s="10">
         <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="13" t="s">
+      <c r="A7" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="14">
-        <v>1</v>
-      </c>
-      <c r="C7" s="14">
+      <c r="B7" s="10">
+        <v>1</v>
+      </c>
+      <c r="C7" s="10">
         <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="13" t="s">
+      <c r="A8" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="14">
-        <v>1</v>
-      </c>
-      <c r="C8" s="14">
+      <c r="B8" s="10">
+        <v>1</v>
+      </c>
+      <c r="C8" s="10">
         <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="13" t="s">
+      <c r="A9" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="B9" s="14">
-        <v>1</v>
-      </c>
-      <c r="C9" s="14">
+      <c r="B9" s="10">
+        <v>1</v>
+      </c>
+      <c r="C9" s="10">
         <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="13" t="s">
+      <c r="A10" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="14">
-        <v>1</v>
-      </c>
-      <c r="C10" s="14">
+      <c r="B10" s="10">
+        <v>1</v>
+      </c>
+      <c r="C10" s="10">
         <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" s="14" t="s">
+      <c r="A11" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="14">
-        <v>1</v>
-      </c>
-      <c r="C11" s="14">
+      <c r="B11" s="10">
+        <v>1</v>
+      </c>
+      <c r="C11" s="10">
         <v>5</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="14" t="s">
+      <c r="A12" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="14">
-        <v>1</v>
-      </c>
-      <c r="C12" s="14">
+      <c r="B12" s="10">
+        <v>1</v>
+      </c>
+      <c r="C12" s="10">
         <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="14" t="s">
+      <c r="A13" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="B13" s="14">
-        <v>1</v>
-      </c>
-      <c r="C13" s="14">
+      <c r="B13" s="10">
+        <v>1</v>
+      </c>
+      <c r="C13" s="10">
         <v>3</v>
       </c>
     </row>
@@ -1209,16 +1206,15 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4AF8CA8F-1DBE-42B3-8633-48C2ED5062E9}">
   <sheetPr codeName="Sheet6"/>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>14</v>
       </c>
@@ -1226,144 +1222,146 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>29</v>
       </c>
-      <c r="B2" s="8">
-        <v>137010500</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B2" s="12">
+        <v>398056107.80000001</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>34</v>
       </c>
-      <c r="B3" s="8">
-        <v>283717500</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B3" s="12">
+        <f>B4*0.4</f>
+        <v>27888660.208000004</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>32</v>
       </c>
       <c r="B4" s="12">
-        <v>9879500</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+        <v>69721650.520000011</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>13</v>
       </c>
       <c r="B5" s="12">
-        <v>108804000</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+        <v>590379508</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>19</v>
       </c>
-      <c r="B6" s="11">
-        <v>257581400</v>
-      </c>
-      <c r="D6" s="8"/>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B6" s="12">
+        <v>280763726</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>25</v>
       </c>
-      <c r="B7" s="11">
-        <v>837500100</v>
-      </c>
-      <c r="D7" s="10"/>
-      <c r="E7" s="9"/>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B7" s="12">
+        <v>879375105</v>
+      </c>
+      <c r="C7" s="8"/>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>21</v>
       </c>
-      <c r="B8" s="11">
-        <v>78464000</v>
-      </c>
-      <c r="E8" s="9"/>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B8" s="12">
+        <v>83171840</v>
+      </c>
+      <c r="C8" s="8"/>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>39</v>
       </c>
       <c r="B9" s="12">
-        <v>10000000</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="6" t="s">
+        <v>7682600</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="11" t="s">
         <v>40</v>
       </c>
       <c r="B10" s="12">
-        <v>10000000</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="6" t="s">
+        <v>3278988.3000000003</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="11" t="s">
         <v>7</v>
       </c>
       <c r="B11" s="12">
-        <v>10000000</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="6" t="s">
+        <v>2828944.58</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" s="11" t="s">
         <v>41</v>
       </c>
       <c r="B12" s="12">
-        <v>10000000</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="6" t="s">
+        <v>116834378.346</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" s="11" t="s">
         <v>27</v>
       </c>
       <c r="B13" s="12">
-        <v>143856000</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="6" t="s">
+        <v>5298997.5940000033</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" s="11" t="s">
         <v>42</v>
       </c>
       <c r="B14" s="12">
-        <v>10000000</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" s="6" t="s">
+        <f>B15*0.7</f>
+        <v>30290394.386</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" s="11" t="s">
         <v>43</v>
       </c>
       <c r="B15" s="12">
-        <v>10000000</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" s="6" t="s">
+        <f>B16*0.5</f>
+        <v>43271991.980000004</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" s="11" t="s">
         <v>44</v>
       </c>
       <c r="B16" s="12">
-        <v>43714500</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" s="6" t="s">
+        <v>86543983.960000008</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" s="11" t="s">
         <v>9</v>
       </c>
       <c r="B17" s="12">
-        <v>9216211.8592507206</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" s="6" t="s">
+        <v>212278110.00000003</v>
+      </c>
+      <c r="C17" s="7"/>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" s="11" t="s">
         <v>10</v>
       </c>
       <c r="B18" s="12">
-        <v>67456638.140749902</v>
+        <v>151027740</v>
       </c>
     </row>
   </sheetData>
@@ -1393,7 +1391,7 @@
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="7">
+      <c r="B2" s="6">
         <v>109769715.256769</v>
       </c>
     </row>
@@ -1401,7 +1399,7 @@
       <c r="A3" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="7">
+      <c r="B3" s="6">
         <v>76483381.4640522</v>
       </c>
     </row>
@@ -1409,7 +1407,7 @@
       <c r="A4" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="7">
+      <c r="B4" s="6">
         <v>111936141.058823</v>
       </c>
     </row>
@@ -1417,7 +1415,7 @@
       <c r="A5" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B5" s="7">
+      <c r="B5" s="6">
         <v>6763202.4705882296</v>
       </c>
     </row>
@@ -1425,7 +1423,7 @@
       <c r="A6" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B6" s="7">
+      <c r="B6" s="6">
         <v>50081880.540420704</v>
       </c>
     </row>
@@ -1433,7 +1431,7 @@
       <c r="A7" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="7">
+      <c r="B7" s="6">
         <v>59034355.4808589</v>
       </c>
     </row>
@@ -1441,7 +1439,7 @@
       <c r="A8" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="7">
+      <c r="B8" s="6">
         <v>171888397.557423</v>
       </c>
     </row>
@@ -1449,7 +1447,7 @@
       <c r="A9" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="7">
+      <c r="B9" s="6">
         <v>52857961.247619003</v>
       </c>
     </row>
@@ -1457,7 +1455,7 @@
       <c r="A10" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B10" s="7">
+      <c r="B10" s="6">
         <v>63880730.2712842</v>
       </c>
     </row>
@@ -1465,7 +1463,7 @@
       <c r="A11" t="s">
         <v>4</v>
       </c>
-      <c r="B11" s="7">
+      <c r="B11" s="6">
         <v>106632842.278244</v>
       </c>
     </row>
@@ -1473,7 +1471,7 @@
       <c r="A12" t="s">
         <v>6</v>
       </c>
-      <c r="B12" s="7">
+      <c r="B12" s="6">
         <v>148000000</v>
       </c>
     </row>
@@ -1481,7 +1479,7 @@
       <c r="A13" t="s">
         <v>9</v>
       </c>
-      <c r="B13" s="7">
+      <c r="B13" s="6">
         <v>21600000</v>
       </c>
     </row>

</xml_diff>